<commit_message>
Actualización del proyecto: Modificaciones en módulos y limpieza de archivos
</commit_message>
<xml_diff>
--- a/EncuestaCompleta.xlsx
+++ b/EncuestaCompleta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\UOC\SEMESTRE3\PRACTICAS\Proyecto_UES\BD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\UOC\SEMESTRE3\TFM\CENSALUD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B996DED8-2713-4CD4-ADA3-C07D5A20B525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DBC6A6F-08FC-4E1C-B8EA-922B712E67D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{36ED46CA-9055-4704-A388-C3E0624374D2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{36ED46CA-9055-4704-A388-C3E0624374D2}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="155">
   <si>
     <t>ID</t>
   </si>
@@ -513,6 +513,18 @@
   </si>
   <si>
     <t>A_40</t>
+  </si>
+  <si>
+    <t>DENV_1</t>
+  </si>
+  <si>
+    <t>DENV_2</t>
+  </si>
+  <si>
+    <t>DENV_3</t>
+  </si>
+  <si>
+    <t>DENV_4</t>
   </si>
 </sst>
 </file>
@@ -522,7 +534,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/mm/yyyy"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -584,6 +596,11 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="11">
@@ -726,7 +743,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
@@ -829,6 +846,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1145,10 +1165,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCB8F8A1-CB86-44F5-AC68-4908B2CE16F7}">
-  <dimension ref="A1:CI23"/>
+  <dimension ref="A1:CM23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.42578125" style="34" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.140625" customWidth="1"/>
     <col min="4" max="5" width="20.140625" customWidth="1"/>
@@ -1196,7 +1216,7 @@
     <col min="87" max="87" width="7.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87" s="5" customFormat="1" ht="68.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:91" s="5" customFormat="1" ht="68.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1458,8 +1478,20 @@
       <c r="CI1" s="5" t="s">
         <v>36</v>
       </c>
+      <c r="CJ1" s="39" t="s">
+        <v>151</v>
+      </c>
+      <c r="CK1" s="39" t="s">
+        <v>152</v>
+      </c>
+      <c r="CL1" s="39" t="s">
+        <v>153</v>
+      </c>
+      <c r="CM1" s="39" t="s">
+        <v>154</v>
+      </c>
     </row>
-    <row r="2" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>37</v>
       </c>
@@ -1721,8 +1753,20 @@
       <c r="CI2" s="9">
         <v>0</v>
       </c>
+      <c r="CJ2">
+        <v>1</v>
+      </c>
+      <c r="CK2">
+        <v>0</v>
+      </c>
+      <c r="CL2">
+        <v>1</v>
+      </c>
+      <c r="CM2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>42</v>
       </c>
@@ -1984,8 +2028,20 @@
       <c r="CI3" s="9">
         <v>0</v>
       </c>
+      <c r="CJ3">
+        <v>1</v>
+      </c>
+      <c r="CK3">
+        <v>0</v>
+      </c>
+      <c r="CL3">
+        <v>1</v>
+      </c>
+      <c r="CM3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
@@ -2247,8 +2303,20 @@
       <c r="CI4" s="9">
         <v>0</v>
       </c>
+      <c r="CJ4">
+        <v>1</v>
+      </c>
+      <c r="CK4">
+        <v>1</v>
+      </c>
+      <c r="CL4">
+        <v>1</v>
+      </c>
+      <c r="CM4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>46</v>
       </c>
@@ -2510,8 +2578,20 @@
       <c r="CI5" s="9">
         <v>0</v>
       </c>
+      <c r="CJ5">
+        <v>0</v>
+      </c>
+      <c r="CK5">
+        <v>0</v>
+      </c>
+      <c r="CL5">
+        <v>1</v>
+      </c>
+      <c r="CM5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>49</v>
       </c>
@@ -2773,8 +2853,20 @@
       <c r="CI6" s="9">
         <v>1</v>
       </c>
+      <c r="CJ6">
+        <v>0</v>
+      </c>
+      <c r="CK6">
+        <v>0</v>
+      </c>
+      <c r="CL6">
+        <v>1</v>
+      </c>
+      <c r="CM6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>52</v>
       </c>
@@ -3036,8 +3128,20 @@
       <c r="CI7" s="9">
         <v>0</v>
       </c>
+      <c r="CJ7">
+        <v>1</v>
+      </c>
+      <c r="CK7">
+        <v>1</v>
+      </c>
+      <c r="CL7">
+        <v>0</v>
+      </c>
+      <c r="CM7">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>54</v>
       </c>
@@ -3299,8 +3403,20 @@
       <c r="CI8" s="9">
         <v>0</v>
       </c>
+      <c r="CJ8">
+        <v>0</v>
+      </c>
+      <c r="CK8">
+        <v>0</v>
+      </c>
+      <c r="CL8">
+        <v>0</v>
+      </c>
+      <c r="CM8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>57</v>
       </c>
@@ -3562,8 +3678,20 @@
       <c r="CI9" s="9">
         <v>1</v>
       </c>
+      <c r="CJ9">
+        <v>0</v>
+      </c>
+      <c r="CK9">
+        <v>1</v>
+      </c>
+      <c r="CL9">
+        <v>0</v>
+      </c>
+      <c r="CM9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>60</v>
       </c>
@@ -3825,8 +3953,20 @@
       <c r="CI10" s="9">
         <v>0</v>
       </c>
+      <c r="CJ10">
+        <v>0</v>
+      </c>
+      <c r="CK10">
+        <v>0</v>
+      </c>
+      <c r="CL10">
+        <v>1</v>
+      </c>
+      <c r="CM10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:91" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>63</v>
       </c>
@@ -4088,8 +4228,20 @@
       <c r="CI11" s="9">
         <v>0</v>
       </c>
+      <c r="CJ11">
+        <v>1</v>
+      </c>
+      <c r="CK11">
+        <v>0</v>
+      </c>
+      <c r="CL11">
+        <v>1</v>
+      </c>
+      <c r="CM11">
+        <v>1</v>
+      </c>
     </row>
-    <row r="12" spans="1:87" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:91" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>65</v>
       </c>
@@ -4351,13 +4503,25 @@
       <c r="CI12" s="9">
         <v>0</v>
       </c>
+      <c r="CJ12">
+        <v>1</v>
+      </c>
+      <c r="CK12">
+        <v>1</v>
+      </c>
+      <c r="CL12">
+        <v>1</v>
+      </c>
+      <c r="CM12">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>67</v>
       </c>
       <c r="B13" s="33">
-        <v>45503</v>
+        <v>45474</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>68</v>
@@ -4614,13 +4778,25 @@
       <c r="CI13" s="20">
         <v>1</v>
       </c>
+      <c r="CJ13">
+        <v>0</v>
+      </c>
+      <c r="CK13">
+        <v>0</v>
+      </c>
+      <c r="CL13">
+        <v>0</v>
+      </c>
+      <c r="CM13">
+        <v>1</v>
+      </c>
     </row>
-    <row r="14" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
         <v>71</v>
       </c>
       <c r="B14" s="33">
-        <v>45503</v>
+        <v>45480</v>
       </c>
       <c r="C14" s="18" t="s">
         <v>68</v>
@@ -4877,13 +5053,25 @@
       <c r="CI14" s="20">
         <v>0</v>
       </c>
+      <c r="CJ14">
+        <v>0</v>
+      </c>
+      <c r="CK14">
+        <v>0</v>
+      </c>
+      <c r="CL14">
+        <v>1</v>
+      </c>
+      <c r="CM14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
         <v>74</v>
       </c>
       <c r="B15" s="33">
-        <v>45503</v>
+        <v>45487</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>68</v>
@@ -5140,13 +5328,25 @@
       <c r="CI15" s="20" t="s">
         <v>41</v>
       </c>
+      <c r="CJ15">
+        <v>1</v>
+      </c>
+      <c r="CK15">
+        <v>1</v>
+      </c>
+      <c r="CL15">
+        <v>1</v>
+      </c>
+      <c r="CM15">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
         <v>77</v>
       </c>
       <c r="B16" s="33">
-        <v>45503</v>
+        <v>45494</v>
       </c>
       <c r="C16" s="18" t="s">
         <v>68</v>
@@ -5403,8 +5603,20 @@
       <c r="CI16" s="20">
         <v>0</v>
       </c>
+      <c r="CJ16">
+        <v>1</v>
+      </c>
+      <c r="CK16">
+        <v>0</v>
+      </c>
+      <c r="CL16">
+        <v>0</v>
+      </c>
+      <c r="CM16">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
         <v>80</v>
       </c>
@@ -5666,8 +5878,20 @@
       <c r="CI17" s="20">
         <v>1</v>
       </c>
+      <c r="CJ17">
+        <v>0</v>
+      </c>
+      <c r="CK17">
+        <v>1</v>
+      </c>
+      <c r="CL17">
+        <v>1</v>
+      </c>
+      <c r="CM17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="18" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>82</v>
       </c>
@@ -5929,8 +6153,20 @@
       <c r="CI18" s="20">
         <v>0</v>
       </c>
+      <c r="CJ18">
+        <v>1</v>
+      </c>
+      <c r="CK18">
+        <v>0</v>
+      </c>
+      <c r="CL18">
+        <v>1</v>
+      </c>
+      <c r="CM18">
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
         <v>84</v>
       </c>
@@ -6192,8 +6428,20 @@
       <c r="CI19" s="20">
         <v>1</v>
       </c>
+      <c r="CJ19">
+        <v>1</v>
+      </c>
+      <c r="CK19">
+        <v>1</v>
+      </c>
+      <c r="CL19">
+        <v>1</v>
+      </c>
+      <c r="CM19">
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
         <v>86</v>
       </c>
@@ -6455,8 +6703,20 @@
       <c r="CI20" s="20">
         <v>0</v>
       </c>
+      <c r="CJ20">
+        <v>1</v>
+      </c>
+      <c r="CK20">
+        <v>0</v>
+      </c>
+      <c r="CL20">
+        <v>0</v>
+      </c>
+      <c r="CM20">
+        <v>1</v>
+      </c>
     </row>
-    <row r="21" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
         <v>89</v>
       </c>
@@ -6718,8 +6978,20 @@
       <c r="CI21" s="20">
         <v>0</v>
       </c>
+      <c r="CJ21">
+        <v>0</v>
+      </c>
+      <c r="CK21">
+        <v>1</v>
+      </c>
+      <c r="CL21">
+        <v>1</v>
+      </c>
+      <c r="CM21">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:87" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:91" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
         <v>91</v>
       </c>
@@ -6981,8 +7253,20 @@
       <c r="CI22" s="20">
         <v>1</v>
       </c>
+      <c r="CJ22">
+        <v>0</v>
+      </c>
+      <c r="CK22">
+        <v>0</v>
+      </c>
+      <c r="CL22">
+        <v>1</v>
+      </c>
+      <c r="CM22">
+        <v>0</v>
+      </c>
     </row>
-    <row r="23" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:91" x14ac:dyDescent="0.25">
       <c r="CD23" s="24"/>
       <c r="CE23" s="35"/>
     </row>

</xml_diff>